<commit_message>
Timing Summary; closes #1206
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/timing/TimingStats_da.xlsx
+++ b/owlcms/src/main/resources/templates/timing/TimingStats_da.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\timing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC2F61F7-06BA-40A3-9D64-BA0D507F03F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E880C6D-6312-434B-80F7-8259CED0355A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3840" yWindow="2805" windowWidth="21600" windowHeight="11295"/>
+    <workbookView xWindow="-26805" yWindow="3135" windowWidth="26610" windowHeight="13980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Données" sheetId="1" r:id="rId1"/>
@@ -54,16 +54,7 @@
     <definedName name="TAS">Données!#REF!</definedName>
     <definedName name="tirage">Données!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="145621" fullCalcOnLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="145621"/>
 </workbook>
 </file>
 
@@ -172,26 +163,26 @@
     <t>${s.athletesPerHour}</t>
   </si>
   <si>
-    <t>$[if(f8 &gt; 0,f8/h8,"")]</t>
-  </si>
-  <si>
     <t>Varighed pr forsøg</t>
   </si>
   <si>
     <t>&lt;jx:forEach items="${groupStats}" var="s"&gt;</t>
+  </si>
+  <si>
+    <t>${s.cJBreakSeconds}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="6">
-    <numFmt numFmtId="186" formatCode="0.0;;"/>
-    <numFmt numFmtId="188" formatCode="_-#,##0;[Red]\(#,##0\);\-"/>
-    <numFmt numFmtId="195" formatCode="0;\(0\);\-"/>
-    <numFmt numFmtId="201" formatCode="0\ ;\(0\)\ ;\-\ "/>
-    <numFmt numFmtId="204" formatCode="0;;"/>
-    <numFmt numFmtId="205" formatCode="[h]:mm:ss;@"/>
+    <numFmt numFmtId="164" formatCode="0.0;;"/>
+    <numFmt numFmtId="165" formatCode="_-#,##0;[Red]\(#,##0\);\-"/>
+    <numFmt numFmtId="166" formatCode="0;\(0\);\-"/>
+    <numFmt numFmtId="167" formatCode="0\ ;\(0\)\ ;\-\ "/>
+    <numFmt numFmtId="168" formatCode="0;;"/>
+    <numFmt numFmtId="169" formatCode="[h]:mm:ss;@"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -489,94 +480,74 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="195" fontId="14" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="188" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="201" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -584,11 +555,11 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -597,39 +568,31 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="186" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="204" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="205" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -644,17 +607,17 @@
     <cellStyle name="Accent4" xfId="4" builtinId="41" customBuiltin="1"/>
     <cellStyle name="Accent5" xfId="5" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Accent6" xfId="6" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Emphase 1" xfId="7"/>
-    <cellStyle name="Emphase 2" xfId="8"/>
-    <cellStyle name="Emphase 3" xfId="9"/>
-    <cellStyle name="Lien hypertexte 2" xfId="10"/>
+    <cellStyle name="Emphase 1" xfId="7" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Emphase 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Emphase 3" xfId="9" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Lien hypertexte 2" xfId="10" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="11"/>
-    <cellStyle name="Normal 3" xfId="12"/>
-    <cellStyle name="Titre 1" xfId="13"/>
-    <cellStyle name="Titre 1 1" xfId="14"/>
-    <cellStyle name="Titre 1 1 1" xfId="15"/>
-    <cellStyle name="Titre de la feuille" xfId="16"/>
+    <cellStyle name="Normal 2" xfId="11" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+    <cellStyle name="Normal 3" xfId="12" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
+    <cellStyle name="Titre 1" xfId="13" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
+    <cellStyle name="Titre 1 1" xfId="14" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
+    <cellStyle name="Titre 1 1 1" xfId="15" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
+    <cellStyle name="Titre de la feuille" xfId="16" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="1">
@@ -1033,11 +996,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Feuil4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y101"/>
+  <dimension ref="A1:X101"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.42578125" customWidth="1"/>
@@ -1045,25 +1008,25 @@
     <col min="3" max="3" width="26.85546875" customWidth="1"/>
     <col min="4" max="4" width="26.140625" customWidth="1"/>
     <col min="5" max="5" width="1.42578125" style="1" hidden="1" customWidth="1"/>
-    <col min="6" max="7" width="12.28515625" style="2" customWidth="1"/>
+    <col min="6" max="7" width="12.28515625" style="1" customWidth="1"/>
     <col min="8" max="8" width="10.42578125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" style="2" customWidth="1"/>
     <col min="10" max="10" width="12.42578125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="16.28515625" style="29" customWidth="1"/>
+    <col min="11" max="11" width="16.28515625" style="21" customWidth="1"/>
     <col min="12" max="13" width="7.7109375" style="1" customWidth="1"/>
     <col min="14" max="14" width="7.7109375" customWidth="1"/>
-    <col min="15" max="15" width="7.7109375" style="4" customWidth="1"/>
+    <col min="15" max="15" width="7.7109375" style="3" customWidth="1"/>
     <col min="16" max="16" width="9.7109375" style="1" customWidth="1"/>
     <col min="17" max="18" width="7.7109375" style="1" customWidth="1"/>
     <col min="19" max="19" width="7.7109375" customWidth="1"/>
-    <col min="20" max="21" width="7.7109375" style="2" customWidth="1"/>
+    <col min="20" max="21" width="7.7109375" style="1" customWidth="1"/>
     <col min="22" max="22" width="6.28515625" style="1" customWidth="1"/>
     <col min="23" max="23" width="4.140625" style="1" customWidth="1"/>
-    <col min="24" max="24" width="8.140625" style="2" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="1" style="5" customWidth="1"/>
+    <col min="24" max="24" width="8.140625" style="1" hidden="1" customWidth="1"/>
+    <col min="25" max="25" width="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="6" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" ht="6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1079,13 +1042,13 @@
       <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -1094,539 +1057,520 @@
       <c r="J1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="29" t="s">
+      <c r="K1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="4"/>
+      <c r="L1" s="3"/>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
       <c r="P1"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
       <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="V1" s="5"/>
+      <c r="V1"/>
       <c r="W1"/>
       <c r="X1"/>
-      <c r="Y1"/>
-    </row>
-    <row r="2" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="35"/>
-      <c r="B2" s="11" t="s">
+    </row>
+    <row r="2" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="27"/>
+      <c r="B2" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="7"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="30"/>
-      <c r="L2" s="4"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="22"/>
+      <c r="L2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
       <c r="P2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2"/>
       <c r="S2" s="1"/>
-      <c r="T2" s="1"/>
-      <c r="V2" s="5"/>
+      <c r="V2"/>
       <c r="W2"/>
       <c r="X2"/>
-      <c r="Y2"/>
-    </row>
-    <row r="3" spans="1:25" ht="14.25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:24" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="36" t="s">
+      <c r="C3" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="12"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13" t="s">
+      <c r="D3" s="9"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="H3" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="37" t="s">
+      <c r="I3" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="30"/>
-      <c r="L3" s="4"/>
+      <c r="J3" s="22"/>
+      <c r="L3" s="3"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
       <c r="P3"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
       <c r="S3" s="1"/>
-      <c r="T3" s="1"/>
-      <c r="V3" s="5"/>
+      <c r="V3"/>
       <c r="W3"/>
       <c r="X3"/>
-      <c r="Y3"/>
-    </row>
-    <row r="4" spans="1:25" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:24" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="14" t="s">
+      <c r="D4" s="16"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="37" t="s">
+      <c r="I4" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="30"/>
-      <c r="L4" s="4"/>
+      <c r="J4" s="22"/>
+      <c r="L4" s="3"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="P4"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
       <c r="S4" s="1"/>
-      <c r="T4" s="1"/>
-      <c r="V4" s="5"/>
+      <c r="V4"/>
       <c r="W4"/>
       <c r="X4"/>
-      <c r="Y4"/>
-    </row>
-    <row r="5" spans="1:25" s="23" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="23" t="s">
+    </row>
+    <row r="5" spans="1:24" s="17" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="50" t="s">
+      <c r="B5" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="50"/>
-      <c r="J5" s="50"/>
-      <c r="K5" s="50"/>
-      <c r="L5" s="24"/>
-      <c r="M5" s="25"/>
-      <c r="N5" s="25"/>
-      <c r="O5" s="25"/>
-      <c r="Q5" s="26"/>
-      <c r="R5" s="26"/>
-      <c r="S5" s="25"/>
-      <c r="T5" s="25"/>
-      <c r="U5" s="26"/>
-      <c r="V5" s="27"/>
-    </row>
-    <row r="6" spans="1:25" s="15" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="28"/>
-      <c r="B6" s="39" t="s">
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
+      <c r="K5" s="40"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+    </row>
+    <row r="6" spans="1:24" s="1" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A6" s="20"/>
+      <c r="B6" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="40" t="s">
+      <c r="E6" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="F6" s="41" t="s">
+      <c r="F6" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="41" t="s">
+      <c r="G6" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="43" t="s">
+      <c r="H6" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="45" t="s">
+      <c r="I6" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="J6" s="43" t="s">
+      <c r="J6" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="11"/>
+    </row>
+    <row r="7" spans="1:24" s="15" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="K6" s="16"/>
-      <c r="L6" s="21"/>
-    </row>
-    <row r="7" spans="1:25" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="34" t="s">
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="25"/>
+      <c r="J7" s="25"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="14"/>
+    </row>
+    <row r="8" spans="1:24" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="20"/>
+      <c r="B8" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="I8" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="J8" s="39" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="33"/>
-      <c r="I7" s="33"/>
-      <c r="J7" s="33"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="19"/>
-    </row>
-    <row r="8" spans="1:25" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="28"/>
-      <c r="B8" s="39" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="48" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="48" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="40" t="s">
-        <v>0</v>
-      </c>
-      <c r="F8" s="49" t="s">
-        <v>31</v>
-      </c>
-      <c r="G8" s="44" t="s">
-        <v>32</v>
-      </c>
-      <c r="H8" s="42" t="s">
-        <v>10</v>
-      </c>
-      <c r="I8" s="46" t="s">
-        <v>33</v>
-      </c>
-      <c r="J8" s="49" t="s">
-        <v>34</v>
-      </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="21"/>
-    </row>
-    <row r="9" spans="1:25" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="34" t="s">
+      <c r="K8" s="11"/>
+    </row>
+    <row r="9" spans="1:24" s="15" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="33"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="33"/>
-      <c r="K9" s="29"/>
-      <c r="L9" s="18"/>
-      <c r="M9" s="19"/>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="B9" s="25"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="25"/>
+      <c r="K9" s="21"/>
+      <c r="L9" s="13"/>
+      <c r="M9" s="14"/>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="2"/>
-      <c r="F10" s="49" t="s">
+      <c r="D10" s="1"/>
+      <c r="F10" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="47" t="s">
+      <c r="G10" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="46" t="s">
+      <c r="H10" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="I10" s="46" t="s">
+      <c r="I10" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="J10" s="49" t="s">
+      <c r="J10" s="39" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="D12" s="2"/>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="D14" s="2"/>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="D15" s="2"/>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="D16" s="2"/>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="D11" s="1"/>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="D16" s="1"/>
     </row>
     <row r="17" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D17" s="2"/>
+      <c r="D17" s="1"/>
     </row>
     <row r="18" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D18" s="2"/>
+      <c r="D18" s="1"/>
     </row>
     <row r="19" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D19" s="2"/>
+      <c r="D19" s="1"/>
     </row>
     <row r="20" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D20" s="2"/>
+      <c r="D20" s="1"/>
     </row>
     <row r="21" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D21" s="2"/>
+      <c r="D21" s="1"/>
     </row>
     <row r="22" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D22" s="2"/>
+      <c r="D22" s="1"/>
     </row>
     <row r="23" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D23" s="2"/>
+      <c r="D23" s="1"/>
     </row>
     <row r="24" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D24" s="2"/>
+      <c r="D24" s="1"/>
     </row>
     <row r="25" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D25" s="2"/>
+      <c r="D25" s="1"/>
     </row>
     <row r="26" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D26" s="2"/>
+      <c r="D26" s="1"/>
     </row>
     <row r="27" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D27" s="2"/>
+      <c r="D27" s="1"/>
     </row>
     <row r="28" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D28" s="2"/>
+      <c r="D28" s="1"/>
     </row>
     <row r="29" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D29" s="2"/>
+      <c r="D29" s="1"/>
     </row>
     <row r="30" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D30" s="2"/>
+      <c r="D30" s="1"/>
     </row>
     <row r="31" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D31" s="2"/>
+      <c r="D31" s="1"/>
     </row>
     <row r="32" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D32" s="2"/>
+      <c r="D32" s="1"/>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D33" s="2"/>
+      <c r="D33" s="1"/>
     </row>
     <row r="34" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D34" s="2"/>
+      <c r="D34" s="1"/>
     </row>
     <row r="35" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D35" s="2"/>
+      <c r="D35" s="1"/>
     </row>
     <row r="36" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D36" s="2"/>
+      <c r="D36" s="1"/>
     </row>
     <row r="37" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D37" s="2"/>
+      <c r="D37" s="1"/>
     </row>
     <row r="38" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D38" s="2"/>
+      <c r="D38" s="1"/>
     </row>
     <row r="39" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D39" s="2"/>
+      <c r="D39" s="1"/>
     </row>
     <row r="40" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D40" s="2"/>
+      <c r="D40" s="1"/>
     </row>
     <row r="41" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D41" s="2"/>
+      <c r="D41" s="1"/>
     </row>
     <row r="42" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D42" s="2"/>
+      <c r="D42" s="1"/>
     </row>
     <row r="43" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D43" s="2"/>
+      <c r="D43" s="1"/>
     </row>
     <row r="44" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D44" s="2"/>
+      <c r="D44" s="1"/>
     </row>
     <row r="45" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D45" s="2"/>
+      <c r="D45" s="1"/>
     </row>
     <row r="46" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D46" s="2"/>
+      <c r="D46" s="1"/>
     </row>
     <row r="47" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D47" s="2"/>
+      <c r="D47" s="1"/>
     </row>
     <row r="48" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D48" s="2"/>
+      <c r="D48" s="1"/>
     </row>
     <row r="49" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D49" s="2"/>
+      <c r="D49" s="1"/>
     </row>
     <row r="50" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D50" s="2"/>
+      <c r="D50" s="1"/>
     </row>
     <row r="51" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D51" s="2"/>
+      <c r="D51" s="1"/>
     </row>
     <row r="52" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D52" s="2"/>
+      <c r="D52" s="1"/>
     </row>
     <row r="53" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D53" s="2"/>
+      <c r="D53" s="1"/>
     </row>
     <row r="54" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D54" s="2"/>
+      <c r="D54" s="1"/>
     </row>
     <row r="55" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D55" s="2"/>
+      <c r="D55" s="1"/>
     </row>
     <row r="56" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D56" s="2"/>
+      <c r="D56" s="1"/>
     </row>
     <row r="57" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D57" s="2"/>
+      <c r="D57" s="1"/>
     </row>
     <row r="58" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D58" s="2"/>
+      <c r="D58" s="1"/>
     </row>
     <row r="59" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D59" s="2"/>
+      <c r="D59" s="1"/>
     </row>
     <row r="60" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D60" s="2"/>
+      <c r="D60" s="1"/>
     </row>
     <row r="61" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D61" s="2"/>
+      <c r="D61" s="1"/>
     </row>
     <row r="62" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D62" s="2"/>
+      <c r="D62" s="1"/>
     </row>
     <row r="63" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D63" s="2"/>
+      <c r="D63" s="1"/>
     </row>
     <row r="64" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D64" s="2"/>
+      <c r="D64" s="1"/>
     </row>
     <row r="65" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D65" s="2"/>
+      <c r="D65" s="1"/>
     </row>
     <row r="66" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D66" s="2"/>
+      <c r="D66" s="1"/>
     </row>
     <row r="67" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D67" s="2"/>
+      <c r="D67" s="1"/>
     </row>
     <row r="68" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D68" s="2"/>
+      <c r="D68" s="1"/>
     </row>
     <row r="69" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D69" s="2"/>
+      <c r="D69" s="1"/>
     </row>
     <row r="70" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D70" s="2"/>
+      <c r="D70" s="1"/>
     </row>
     <row r="71" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D71" s="2"/>
+      <c r="D71" s="1"/>
     </row>
     <row r="72" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D72" s="2"/>
+      <c r="D72" s="1"/>
     </row>
     <row r="73" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D73" s="2"/>
+      <c r="D73" s="1"/>
     </row>
     <row r="74" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D74" s="2"/>
+      <c r="D74" s="1"/>
     </row>
     <row r="75" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D75" s="2"/>
+      <c r="D75" s="1"/>
     </row>
     <row r="76" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D76" s="2"/>
+      <c r="D76" s="1"/>
     </row>
     <row r="77" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D77" s="2"/>
+      <c r="D77" s="1"/>
     </row>
     <row r="78" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D78" s="2"/>
+      <c r="D78" s="1"/>
     </row>
     <row r="79" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D79" s="2"/>
+      <c r="D79" s="1"/>
     </row>
     <row r="80" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D80" s="2"/>
+      <c r="D80" s="1"/>
     </row>
     <row r="81" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D81" s="2"/>
+      <c r="D81" s="1"/>
     </row>
     <row r="82" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D82" s="2"/>
+      <c r="D82" s="1"/>
     </row>
     <row r="83" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D83" s="2"/>
+      <c r="D83" s="1"/>
     </row>
     <row r="84" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D84" s="2"/>
+      <c r="D84" s="1"/>
     </row>
     <row r="85" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D85" s="2"/>
+      <c r="D85" s="1"/>
     </row>
     <row r="86" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D86" s="2"/>
+      <c r="D86" s="1"/>
     </row>
     <row r="87" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D87" s="2"/>
+      <c r="D87" s="1"/>
     </row>
     <row r="88" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D88" s="2"/>
+      <c r="D88" s="1"/>
     </row>
     <row r="89" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D89" s="2"/>
+      <c r="D89" s="1"/>
     </row>
     <row r="90" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D90" s="2"/>
+      <c r="D90" s="1"/>
     </row>
     <row r="91" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D91" s="2"/>
+      <c r="D91" s="1"/>
     </row>
     <row r="92" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D92" s="2"/>
+      <c r="D92" s="1"/>
     </row>
     <row r="93" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D93" s="2"/>
+      <c r="D93" s="1"/>
     </row>
     <row r="94" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D94" s="2"/>
+      <c r="D94" s="1"/>
     </row>
     <row r="95" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D95" s="2"/>
+      <c r="D95" s="1"/>
     </row>
     <row r="96" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D96" s="2"/>
+      <c r="D96" s="1"/>
     </row>
     <row r="97" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D97" s="2"/>
+      <c r="D97" s="1"/>
     </row>
     <row r="98" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D98" s="2"/>
+      <c r="D98" s="1"/>
     </row>
     <row r="99" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D99" s="2"/>
+      <c r="D99" s="1"/>
     </row>
     <row r="100" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D100" s="2"/>
+      <c r="D100" s="1"/>
     </row>
     <row r="101" spans="4:4" x14ac:dyDescent="0.2">
-      <c r="D101" s="2"/>
+      <c r="D101" s="1"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
@@ -1639,7 +1583,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J7">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J7" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0</formula1>
       <formula2>200</formula2>
     </dataValidation>

</xml_diff>